<commit_message>
daily auto-refresh 2026-10-23 06:35
</commit_message>
<xml_diff>
--- a/refundable_samples_rollup.xlsx
+++ b/refundable_samples_rollup.xlsx
@@ -6230,16 +6230,16 @@
         <v>40</v>
       </c>
       <c r="C87">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D87">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E87">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F87">
-        <v>6278.84</v>
+        <v>6318.83</v>
       </c>
       <c r="G87">
         <v>7</v>
@@ -6287,7 +6287,7 @@
         <v>0.6</v>
       </c>
       <c r="V87">
-        <v>6150.66</v>
+        <v>6190.65</v>
       </c>
     </row>
     <row r="88" spans="1:22">
@@ -6298,16 +6298,16 @@
         <v>40</v>
       </c>
       <c r="C88">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="D88">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="E88">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="F88">
-        <v>5318.58</v>
+        <v>5518.33</v>
       </c>
       <c r="G88">
         <v>2</v>
@@ -6343,10 +6343,10 @@
         <v>61</v>
       </c>
       <c r="R88">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="S88">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="T88">
         <v>0</v>
@@ -6355,7 +6355,7 @@
         <v>0</v>
       </c>
       <c r="V88">
-        <v>5303.65</v>
+        <v>5503.4</v>
       </c>
     </row>
     <row r="89" spans="1:22">
@@ -10246,16 +10246,16 @@
         <v>48</v>
       </c>
       <c r="C148">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D148">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E148">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F148">
-        <v>122.98</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="G148">
         <v>0</v>
@@ -10297,7 +10297,7 @@
         <v>0</v>
       </c>
       <c r="V148">
-        <v>122.98</v>
+        <v>82.98999999999999</v>
       </c>
     </row>
     <row r="149" spans="1:22">
@@ -10308,16 +10308,16 @@
         <v>48</v>
       </c>
       <c r="C149">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D149">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E149">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F149">
-        <v>346.41</v>
+        <v>146.66</v>
       </c>
       <c r="G149">
         <v>0</v>
@@ -10359,7 +10359,7 @@
         <v>0</v>
       </c>
       <c r="V149">
-        <v>346.41</v>
+        <v>146.66</v>
       </c>
     </row>
     <row r="150" spans="1:22">

</xml_diff>